<commit_message>
docs(handover): PO rulings D-01..D-12 applied — launch scope register + phased execution plan
- LAUNCH_SCOPE_REGISTER: definitive scope (verified / under remediation /
  approved-for-build / PO-ratified exclusions)
- PHASED_EXECUTION_PLAN: phase gates, dependencies (G-05 before new admin
  surfaces, vendor-auth sign-off before D-01 build, sandbox keys before D-05),
  effort sizing
- Registers/guide/checklist/dashboard regenerated: 'excluded or under
  implementation' replaces 'pending decision'
- Vendor tenancy confirmed: platform-global vendors, tenant-scoped bookings
  (preserved per PO direction)

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/afruheritage-platform/uat-package/AFRUHERITAGE_UAT_CHECKLIST.xlsx
+++ b/afruheritage-platform/uat-package/AFRUHERITAGE_UAT_CHECKLIST.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Checklist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending PO Decision" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Exclusions" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Types" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
@@ -1816,7 +1816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1860,188 +1860,210 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-01)</t>
+          <t>Under implementation (D-01) — not yet deployed</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>The vendor backend lifecycle is already built; the vendor-facing pages are missing. Awaiting a Product Owner decision on marketplace launch scope. Do not test.</t>
+          <t>Approved for build: vendor registration, approval, marketplace bookings. Not yet usable — do not test.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Driver portal (driver sign-in)</t>
+          <t>Central Afruheritage platform support intake</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Fleet management</t>
+          <t>/support on the main site</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-02)</t>
+          <t>Under implementation (D-04)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Drivers are managed records today and cannot sign in. Awaiting decision on whether managed records suffice for launch.</t>
+          <t>A platform-level support channel is being built. Today, tickets are submitted on each company's portal page.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Warehouse operations module</t>
+          <t>CRM activity history</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Not in customer navigation</t>
+          <t>CRM section — contacts and quotes available</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-06)</t>
+          <t>Under implementation (D-08)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>No implementation exists. Awaiting decision: build it, or remove it from the offering.</t>
+          <t>The activity interface is being added. Contacts and quotes already work.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Dedicated analytics dashboards</t>
+          <t>Live payment collection</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Not in customer navigation</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-07)</t>
+          <t>Pending sandbox certification (D-05)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Basic operational counts already work. Awaiting decision on whether basic counts suffice for launch.</t>
+          <t>Manual-renewal billing model — there are no automatic recurring charges. Plan/trial selection works; do not attempt real-money payments during UAT.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CRM activity history</t>
+          <t>Driver portal (driver sign-in)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CRM section — contacts and quotes available</t>
+          <t>Fleet management</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-08)</t>
+          <t>Excluded from initial launch (D-02)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Activity endpoints exist but have no UI. Awaiting decision on launch requirement.</t>
+          <t>Drivers are managed records — creation and assignment work; drivers cannot sign in.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Central support tickets on afruheritage.com</t>
+          <t>Warehouse operations</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>/support on the main site</t>
+          <t>Not in customer navigation</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-04)</t>
+          <t>Excluded from offering (D-06)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Tickets today are submitted on each company's portal. Awaiting decision on a platform-level intake channel.</t>
+          <t>Not part of the Afruheritage launch product.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Additional storefront templates (mall, ecommerce, restaurant, bookings, real estate)</t>
+          <t>Dedicated analytics dashboards</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Templates page</t>
+          <t>Not in customer navigation</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-09)</t>
+          <t>Excluded from initial launch (D-07)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Preview only — publish-blocked until tenant-configurable content is complete.</t>
+          <t>Basic operational counts already work; advanced dashboards follow later.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Mobile app (iOS/Android)</t>
+          <t>Additional storefront templates (mall, ecommerce, restaurant, bookings, real estate)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Templates page</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-11)</t>
+          <t>Excluded — publish-blocked (D-09)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>On the roadmap — the web app works on mobile browsers today.</t>
+          <t>Preview only; cannot be published until tenant-configurable content is complete.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Payment collection (live billing charges)</t>
+          <t>Custom domains</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pending PO decision (D-05)</t>
+          <t>Excluded from initial launch (D-10)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Paystack/Flutterwave integrations exist but are unverified end-to-end. Plan/trial selection works; do not attempt real-money payments during UAT.</t>
+          <t>Company portals run on yourname.afruheritage.com. Custom domains need separate DNS/certificate work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Mobile app (iOS/Android)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Excluded from initial launch (D-11)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>The web app works on mobile browsers; native apps are on the roadmap.</t>
         </is>
       </c>
     </row>

</xml_diff>